<commit_message>
minor edits. correction to spreadsheet
</commit_message>
<xml_diff>
--- a/Quality Improvement Measures vs Billing.xlsx
+++ b/Quality Improvement Measures vs Billing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://spurafrika.sharepoint.com/sites/SlowMedicine/Shared Documents/General/Documents/Quality and Billing/QIMs and Billing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1884" documentId="11_0A83C39547C27BA4B3B8F7925C3BD5758203E6F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA9D8AB1-3680-4F2C-9134-9EA44556A945}"/>
+  <xr:revisionPtr revIDLastSave="1885" documentId="11_0A83C39547C27BA4B3B8F7925C3BD5758203E6F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FF1F9F0-B01A-480E-9CA0-4891CACC640A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6410" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6410" uniqueCount="38">
   <si>
     <t>Time period: July 2024 to Jun 2025</t>
   </si>
@@ -150,9 +150,6 @@
   </si>
   <si>
     <t>Mixed</t>
-  </si>
-  <si>
-    <t>hatrack</t>
   </si>
 </sst>
 </file>
@@ -3234,7 +3231,7 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B120" t="s">
         <v>10</v>

</xml_diff>